<commit_message>
feat: relatorio_td, deepnote skill, AGENTS, gitignore cleanup
- analyses/relatorio_td: novo notebook Deepnote v20260624, regras de negócio,
  formatação de planilha, otimizações de query, governança e README atualizados,
  pipeline SQL atualizado, remoção de td_analysis_functions.py e notebook antigo
- skills/deepnote-notebook: nova skill com SKILL.md, openai.yaml e ícone
- AGENTS.md: adicionado ao repositório
- .gitignore: exclusão de __pycache__, *.pyc e .serena/
- .github/copilot-instructions.md: atualizado
- analytics/lead_time: documentação e dashboard atualizados
</commit_message>
<xml_diff>
--- a/analyses/relatorio_td/TD_Priorizacao_Melhorias_Profissional_20260612.xlsx
+++ b/analyses/relatorio_td/TD_Priorizacao_Melhorias_Profissional_20260612.xlsx
@@ -28,7 +28,7 @@
     <numFmt numFmtId="166" formatCode="R$ #,##0"/>
     <numFmt numFmtId="167" formatCode="0.0"/>
   </numFmts>
-  <fonts count="34">
+  <fonts count="37">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -184,8 +184,22 @@
       <color rgb="00F57F17"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Courier New"/>
+      <color rgb="00212121"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00757575"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <color rgb="00212121"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="23">
+  <fills count="26">
     <fill>
       <patternFill/>
     </fill>
@@ -297,8 +311,23 @@
         <fgColor rgb="00FFF9C4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8F9FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFDE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ECEFF1"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -320,11 +349,55 @@
         <color rgb="00E0E0E0"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00E0E0E0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E0E0E0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E0E0E0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00E0E0E0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E0E0E0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E0E0E0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E0E0E0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E0E0E0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="103">
+  <cellXfs count="110">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -629,6 +702,23 @@
     </xf>
     <xf numFmtId="0" fontId="28" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="23" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="25" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1033,31 +1123,31 @@
           <t>🔴  Priorizar melhoria</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n"/>
+      <c r="B5" s="103" t="n"/>
       <c r="C5" s="5" t="inlineStr">
         <is>
           <t>🟡  Alerta em produto relevante</t>
         </is>
       </c>
-      <c r="D5" s="4" t="n"/>
+      <c r="D5" s="103" t="n"/>
       <c r="E5" s="6" t="inlineStr">
         <is>
           <t>🟠  Monitorar</t>
         </is>
       </c>
-      <c r="F5" s="4" t="n"/>
+      <c r="F5" s="103" t="n"/>
       <c r="G5" s="7" t="inlineStr">
         <is>
           <t>⚪  Não priorizar agora</t>
         </is>
       </c>
-      <c r="H5" s="4" t="n"/>
+      <c r="H5" s="103" t="n"/>
       <c r="I5" s="8" t="inlineStr">
         <is>
           <t>⬜  Sem evidência suficiente</t>
         </is>
       </c>
-      <c r="J5" s="4" t="n"/>
+      <c r="J5" s="103" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
@@ -1385,23 +1475,23 @@
           <t>🔴</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n"/>
+      <c r="B14" s="103" t="n"/>
       <c r="C14" s="13" t="inlineStr">
         <is>
           <t>12 produtos com AÇÃO IMEDIATA</t>
         </is>
       </c>
-      <c r="D14" s="4" t="n"/>
-      <c r="E14" s="4" t="n"/>
+      <c r="D14" s="104" t="n"/>
+      <c r="E14" s="103" t="n"/>
       <c r="F14" s="14" t="inlineStr">
         <is>
           <t>Alta T&amp;D + Alta tração comercial. Concentram 18,6% da receita com 21,8% do volume de T&amp;D.</t>
         </is>
       </c>
-      <c r="G14" s="4" t="n"/>
-      <c r="H14" s="4" t="n"/>
-      <c r="I14" s="4" t="n"/>
-      <c r="J14" s="4" t="n"/>
+      <c r="G14" s="104" t="n"/>
+      <c r="H14" s="104" t="n"/>
+      <c r="I14" s="104" t="n"/>
+      <c r="J14" s="103" t="n"/>
     </row>
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="12" t="inlineStr">
@@ -1409,23 +1499,23 @@
           <t>📍</t>
         </is>
       </c>
-      <c r="B15" s="4" t="n"/>
+      <c r="B15" s="103" t="n"/>
       <c r="C15" s="13" t="inlineStr">
         <is>
           <t>caimento_ruim é o ofensor sistêmico</t>
         </is>
       </c>
-      <c r="D15" s="4" t="n"/>
-      <c r="E15" s="4" t="n"/>
+      <c r="D15" s="104" t="n"/>
+      <c r="E15" s="103" t="n"/>
       <c r="F15" s="14" t="inlineStr">
         <is>
           <t>Presente em 87 produtos; 12 no bucket Priorizar Melhoria. Afeta especialmente Calça, Saia e Cropped femininos.</t>
         </is>
       </c>
-      <c r="G15" s="4" t="n"/>
-      <c r="H15" s="4" t="n"/>
-      <c r="I15" s="4" t="n"/>
-      <c r="J15" s="4" t="n"/>
+      <c r="G15" s="104" t="n"/>
+      <c r="H15" s="104" t="n"/>
+      <c r="I15" s="104" t="n"/>
+      <c r="J15" s="103" t="n"/>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="12" t="inlineStr">
@@ -1433,23 +1523,23 @@
           <t>📈</t>
         </is>
       </c>
-      <c r="B16" s="4" t="n"/>
+      <c r="B16" s="103" t="n"/>
       <c r="C16" s="13" t="inlineStr">
         <is>
           <t>49 produtos com tendência crescente</t>
         </is>
       </c>
-      <c r="D16" s="4" t="n"/>
-      <c r="E16" s="4" t="n"/>
+      <c r="D16" s="104" t="n"/>
+      <c r="E16" s="103" t="n"/>
       <c r="F16" s="14" t="inlineStr">
         <is>
           <t>Reversas aumentaram nos últimos 3 meses vs 3 anteriores. Ação preventiva pode evitar escalada.</t>
         </is>
       </c>
-      <c r="G16" s="4" t="n"/>
-      <c r="H16" s="4" t="n"/>
-      <c r="I16" s="4" t="n"/>
-      <c r="J16" s="4" t="n"/>
+      <c r="G16" s="104" t="n"/>
+      <c r="H16" s="104" t="n"/>
+      <c r="I16" s="104" t="n"/>
+      <c r="J16" s="103" t="n"/>
     </row>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="12" t="inlineStr">
@@ -1457,23 +1547,23 @@
           <t>💰</t>
         </is>
       </c>
-      <c r="B17" s="4" t="n"/>
+      <c r="B17" s="103" t="n"/>
       <c r="C17" s="13" t="inlineStr">
         <is>
           <t>90%+ das reversas são de origem física</t>
         </is>
       </c>
-      <c r="D17" s="4" t="n"/>
-      <c r="E17" s="4" t="n"/>
+      <c r="D17" s="104" t="n"/>
+      <c r="E17" s="103" t="n"/>
       <c r="F17" s="14" t="inlineStr">
         <is>
           <t>Foco de melhoria diretamente no produto — não em logística.</t>
         </is>
       </c>
-      <c r="G17" s="4" t="n"/>
-      <c r="H17" s="4" t="n"/>
-      <c r="I17" s="4" t="n"/>
-      <c r="J17" s="4" t="n"/>
+      <c r="G17" s="104" t="n"/>
+      <c r="H17" s="104" t="n"/>
+      <c r="I17" s="104" t="n"/>
+      <c r="J17" s="103" t="n"/>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="12" t="inlineStr">
@@ -1481,23 +1571,23 @@
           <t>⚠️</t>
         </is>
       </c>
-      <c r="B18" s="4" t="n"/>
+      <c r="B18" s="103" t="n"/>
       <c r="C18" s="13" t="inlineStr">
         <is>
           <t>Produtos KILL com alta T&amp;D confirmada</t>
         </is>
       </c>
-      <c r="D18" s="4" t="n"/>
-      <c r="E18" s="4" t="n"/>
+      <c r="D18" s="104" t="n"/>
+      <c r="E18" s="103" t="n"/>
       <c r="F18" s="14" t="inlineStr">
         <is>
           <t>Calça Studio InLounge Masc., Blusa Manga Longa Comfy, Vestido Sharp InLounge → descontinuação acelerada recomendada.</t>
         </is>
       </c>
-      <c r="G18" s="4" t="n"/>
-      <c r="H18" s="4" t="n"/>
-      <c r="I18" s="4" t="n"/>
-      <c r="J18" s="4" t="n"/>
+      <c r="G18" s="104" t="n"/>
+      <c r="H18" s="104" t="n"/>
+      <c r="I18" s="104" t="n"/>
+      <c r="J18" s="103" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="23">
@@ -15779,11 +15869,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
@@ -15794,14 +15884,14 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="86" t="inlineStr">
         <is>
-          <t>ℹ️  LEGENDA &amp; METODOLOGIA</t>
+          <t>ℹ️  LEGENDA &amp; METODOLOGIA — v2.0 (20/06/2026)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="26" customHeight="1">
       <c r="A3" s="87" t="inlineStr">
         <is>
-          <t>SINAIS DE FAROL</t>
+          <t>SINAIS DE FAROL (sinal_priorizacao)</t>
         </is>
       </c>
     </row>
@@ -15814,7 +15904,7 @@
       <c r="B4" s="4" t="n"/>
       <c r="C4" s="89" t="inlineStr">
         <is>
-          <t>td_score ≥ 0.70 e commercial_score ≥ 0.60  →  Alta dor + Alta tração: ação imediata</t>
+          <t>td_score ≥ 0,70  E  commercial_score_v2 ≥ 0,60  →  Alta dor + alta tração: ação imediata</t>
         </is>
       </c>
       <c r="D4" s="4" t="n"/>
@@ -15825,13 +15915,13 @@
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="90" t="inlineStr">
         <is>
-          <t>🟡 Alerta prod. relevante</t>
+          <t>🟡 Alerta em prod. relevante</t>
         </is>
       </c>
       <c r="B5" s="4" t="n"/>
       <c r="C5" s="89" t="inlineStr">
         <is>
-          <t>commercial_score ≥ 0.70 e td_score ∈ [0.50, 0.70)  →  Produto de peso com dor moderada crescendo</t>
+          <t>commercial_score_v2 ≥ 0,70  E  0,50 ≤ td_score &lt; 0,70  →  Produto de peso com dor moderada em escalada</t>
         </is>
       </c>
       <c r="D5" s="4" t="n"/>
@@ -15848,7 +15938,7 @@
       <c r="B6" s="4" t="n"/>
       <c r="C6" s="89" t="inlineStr">
         <is>
-          <t>td_score ≥ 0.70 e commercial_score &lt; 0.60  →  Alta dor, mas tração insuficiente para priorizar</t>
+          <t>td_score ≥ 0,70  E  commercial_score_v2 &lt; 0,60  →  Alta dor, tração insuficiente  |  OU zona cinza de scores intermediários</t>
         </is>
       </c>
       <c r="D6" s="4" t="n"/>
@@ -15865,7 +15955,7 @@
       <c r="B7" s="4" t="n"/>
       <c r="C7" s="89" t="inlineStr">
         <is>
-          <t>td_score &lt; 0.50 ou commercial_score &lt; 0.40  →  Sem urgência no momento</t>
+          <t>td_score &lt; 0,50  OU  commercial_score_v2 &lt; 0,40  →  Sem urgência no momento</t>
         </is>
       </c>
       <c r="D7" s="4" t="n"/>
@@ -15876,13 +15966,13 @@
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="93" t="inlineStr">
         <is>
-          <t>⬜ Sem evidência</t>
+          <t>⬜ Sem evidência suficiente</t>
         </is>
       </c>
       <c r="B8" s="4" t="n"/>
       <c r="C8" s="89" t="inlineStr">
         <is>
-          <t>&lt; 30 vendas ou &lt; 5 retornos  →  Volume insuficiente para diagnóstico</t>
+          <t>Vendas &lt; 30  OU  retornos &lt; 5  →  Volume insuficiente para diagnóstico confiável</t>
         </is>
       </c>
       <c r="D8" s="4" t="n"/>
@@ -15890,23 +15980,26 @@
       <c r="F8" s="4" t="n"/>
       <c r="G8" s="4" t="n"/>
     </row>
+    <row r="9" ht="6" customHeight="1"/>
     <row r="10" ht="26" customHeight="1">
       <c r="A10" s="87" t="inlineStr">
         <is>
-          <t>SCORES (todos CUME_DIST 0–1 sobre universo de produtos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="94" t="inlineStr">
-        <is>
-          <t>TD Score</t>
+          <t>SCORES  ·  Todos relativos ao portfólio via CUME_DIST() — valor 0,80 = melhor que 80% dos produtos</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="105" t="inlineStr">
+        <is>
+          <t>TD Score  (dor do cliente)</t>
         </is>
       </c>
       <c r="B11" s="4" t="n"/>
-      <c r="C11" s="89" t="inlineStr">
-        <is>
-          <t>0.5 × percentil_td_rate  +  0.3 × percentil_volume_td  +  0.2 × percentil_delta_vs_categoria</t>
+      <c r="C11" s="106" t="inlineStr">
+        <is>
+          <t>td_score = 0,50 × percentil_td_rate
+         + 0,30 × percentil_volume_td
+         + 0,20 × percentil_delta_vs_categoria</t>
         </is>
       </c>
       <c r="D11" s="4" t="n"/>
@@ -15914,16 +16007,17 @@
       <c r="F11" s="4" t="n"/>
       <c r="G11" s="4" t="n"/>
     </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="94" t="inlineStr">
-        <is>
-          <t>Commercial Score</t>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="105" t="inlineStr">
+        <is>
+          <t>Commercial Score v2  (tração + margem)</t>
         </is>
       </c>
       <c r="B12" s="4" t="n"/>
-      <c r="C12" s="89" t="inlineStr">
-        <is>
-          <t>0.6 × percentil_receita  +  0.4 × percentil_unidades</t>
+      <c r="C12" s="106" t="inlineStr">
+        <is>
+          <t>commercial_score_v2 = 0,70 × tracao_vendas_score
+                    + 0,30 × mc3_score</t>
         </is>
       </c>
       <c r="D12" s="4" t="n"/>
@@ -15931,16 +16025,19 @@
       <c r="F12" s="4" t="n"/>
       <c r="G12" s="4" t="n"/>
     </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="94" t="inlineStr">
-        <is>
-          <t>Priority Score</t>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  └─ Bloco 1: tracao_vendas_score  (70%)</t>
         </is>
       </c>
       <c r="B13" s="4" t="n"/>
-      <c r="C13" s="89" t="inlineStr">
-        <is>
-          <t>0.6 × td_score  +  0.4 × commercial_score</t>
+      <c r="C13" s="106" t="inlineStr">
+        <is>
+          <t>tracao_vendas_score = 0,30 × percentil_sell_through_30d
+                    + 0,30 × percentil_sell_through_60d
+                    + 0,25 × percentil_sell_through_90d
+                    + 0,15 × percentil_receita_media_mensal_vs_categoria</t>
         </is>
       </c>
       <c r="D13" s="4" t="n"/>
@@ -15948,40 +16045,61 @@
       <c r="F13" s="4" t="n"/>
       <c r="G13" s="4" t="n"/>
     </row>
-    <row r="15" ht="26" customHeight="1">
-      <c r="A15" s="87" t="inlineStr">
-        <is>
-          <t>CLUSTER ESTRATÉGICO</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="95" t="inlineStr">
-        <is>
-          <t>HERO</t>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ⚠ Fallback (~7 produtos sem estoque): substitui tracao_vendas_score por  0,60 × percentil_receita + 0,40 × percentil_unidades</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n"/>
+      <c r="C14" s="4" t="n"/>
+      <c r="D14" s="4" t="n"/>
+      <c r="E14" s="4" t="n"/>
+      <c r="F14" s="4" t="n"/>
+      <c r="G14" s="4" t="n"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  └─ Bloco 2: mc3_score  (30%)</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="n"/>
+      <c r="C15" s="106" t="inlineStr">
+        <is>
+          <t>mc3_score = 0,50 × mc3_vs_categoria_score    (escala discreta: 1,00 / 0,75 / 0,50 / 0,25)
+          + 0,30 × mc3_vs_portfolio_score     (escala discreta: 1,00 / 0,75 / 0,50 / 0,25)
+          + 0,20 × representatividade_mc3_score  (CUME_DIST sobre net_profit_after_mkt_costs)</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="n"/>
+      <c r="E15" s="4" t="n"/>
+      <c r="F15" s="4" t="n"/>
+      <c r="G15" s="4" t="n"/>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ⚠ Fallback: quando mc3_ratio é NULL (produto ausente em eval_produto_portfolio), commercial_score_v2 = tracao_vendas_score com peso total (1,00). Cobertura atual: ~126/287 produtos.</t>
         </is>
       </c>
       <c r="B16" s="4" t="n"/>
-      <c r="C16" s="89" t="inlineStr">
-        <is>
-          <t>Produto carro-chefe — alta receita e demanda</t>
-        </is>
-      </c>
+      <c r="C16" s="4" t="n"/>
       <c r="D16" s="4" t="n"/>
       <c r="E16" s="4" t="n"/>
       <c r="F16" s="4" t="n"/>
       <c r="G16" s="4" t="n"/>
     </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="96" t="inlineStr">
-        <is>
-          <t>CORE</t>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="105" t="inlineStr">
+        <is>
+          <t>Priority Score  (urgência global)</t>
         </is>
       </c>
       <c r="B17" s="4" t="n"/>
-      <c r="C17" s="89" t="inlineStr">
-        <is>
-          <t>Produto estável e relevante no portfólio</t>
+      <c r="C17" s="106" t="inlineStr">
+        <is>
+          <t>priority_score = 0,50 × td_score  +  0,50 × commercial_score_v2</t>
         </is>
       </c>
       <c r="D17" s="4" t="n"/>
@@ -15989,74 +16107,71 @@
       <c r="F17" s="4" t="n"/>
       <c r="G17" s="4" t="n"/>
     </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="97" t="inlineStr">
-        <is>
-          <t>LONG TAIL</t>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ⚠ Peso igual entre dor do cliente e tração comercial — produto que machuca E tem relevância econômica sobe no ranking.</t>
         </is>
       </c>
       <c r="B18" s="4" t="n"/>
-      <c r="C18" s="89" t="inlineStr">
-        <is>
-          <t>Produto de nicho — volume menor</t>
-        </is>
-      </c>
+      <c r="C18" s="4" t="n"/>
       <c r="D18" s="4" t="n"/>
       <c r="E18" s="4" t="n"/>
       <c r="F18" s="4" t="n"/>
       <c r="G18" s="4" t="n"/>
     </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="98" t="inlineStr">
-        <is>
-          <t>KILL</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="n"/>
-      <c r="C19" s="89" t="inlineStr">
-        <is>
-          <t>Produto marcado para descontinuação</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="n"/>
-      <c r="E19" s="4" t="n"/>
-      <c r="F19" s="4" t="n"/>
-      <c r="G19" s="4" t="n"/>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="99" t="inlineStr">
-        <is>
-          <t>LANCAMENTO</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="n"/>
-      <c r="C20" s="89" t="inlineStr">
-        <is>
-          <t>Produto em ramp-up — commercial_score pode estar subestimado</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="n"/>
-      <c r="E20" s="4" t="n"/>
-      <c r="F20" s="4" t="n"/>
-      <c r="G20" s="4" t="n"/>
-    </row>
-    <row r="22" ht="26" customHeight="1">
-      <c r="A22" s="87" t="inlineStr">
-        <is>
-          <t>TENDÊNCIA (reversas últimos 3m vs 3m anteriores)</t>
-        </is>
-      </c>
+    <row r="19" ht="6" customHeight="1"/>
+    <row r="20" ht="26" customHeight="1">
+      <c r="A20" s="87" t="inlineStr">
+        <is>
+          <t>DECISÃO ESTRATÉGICA (sinal_kill_keep)  ·  Calculado apenas para produtos com evidência suficiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="88" t="inlineStr">
+        <is>
+          <t>🔴 Priorizar melhoria</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="n"/>
+      <c r="C21" s="89" t="inlineStr">
+        <is>
+          <t>td_score ≥ 0,70  E  commercial_score_v2 ≥ 0,60  →  Alta dor + alta tração: investir na correção</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="n"/>
+      <c r="E21" s="4" t="n"/>
+      <c r="F21" s="4" t="n"/>
+      <c r="G21" s="4" t="n"/>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="91" t="inlineStr">
+        <is>
+          <t>🟠 Avaliar Descontinuação / Reformulação</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="n"/>
+      <c r="C22" s="89" t="inlineStr">
+        <is>
+          <t>td_score ≥ 0,70  E  commercial_score_v2 &lt; 0,60  →  Alta dor + baixa tração: avaliar saída do portfólio</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="n"/>
+      <c r="E22" s="4" t="n"/>
+      <c r="F22" s="4" t="n"/>
+      <c r="G22" s="4" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="100" t="inlineStr">
-        <is>
-          <t>Aumentou</t>
+      <c r="A23" s="92" t="inlineStr">
+        <is>
+          <t>⚪ Não priorizar agora</t>
         </is>
       </c>
       <c r="B23" s="4" t="n"/>
       <c r="C23" s="89" t="inlineStr">
         <is>
-          <t>Reversas acelerando — urgência aumentada</t>
+          <t>Demais casos com evidência  →  Sem urgência de decisão estrutural</t>
         </is>
       </c>
       <c r="D23" s="4" t="n"/>
@@ -16064,79 +16179,454 @@
       <c r="F23" s="4" t="n"/>
       <c r="G23" s="4" t="n"/>
     </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="101" t="inlineStr">
+    <row r="24" ht="6" customHeight="1"/>
+    <row r="25" ht="26" customHeight="1">
+      <c r="A25" s="87" t="inlineStr">
+        <is>
+          <t>CLUSTER ESTRATÉGICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="95" t="inlineStr">
+        <is>
+          <t>HERO</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="n"/>
+      <c r="C26" s="89" t="inlineStr">
+        <is>
+          <t>Produto carro-chefe — alta receita e demanda</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="n"/>
+      <c r="E26" s="4" t="n"/>
+      <c r="F26" s="4" t="n"/>
+      <c r="G26" s="4" t="n"/>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="96" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="n"/>
+      <c r="C27" s="89" t="inlineStr">
+        <is>
+          <t>Produto estável e relevante no portfólio</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="n"/>
+      <c r="E27" s="4" t="n"/>
+      <c r="F27" s="4" t="n"/>
+      <c r="G27" s="4" t="n"/>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="97" t="inlineStr">
+        <is>
+          <t>LONG TAIL</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="n"/>
+      <c r="C28" s="89" t="inlineStr">
+        <is>
+          <t>Produto de nicho — volume menor</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="n"/>
+      <c r="E28" s="4" t="n"/>
+      <c r="F28" s="4" t="n"/>
+      <c r="G28" s="4" t="n"/>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="98" t="inlineStr">
+        <is>
+          <t>KILL</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="n"/>
+      <c r="C29" s="89" t="inlineStr">
+        <is>
+          <t>Produto marcado para descontinuação</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="n"/>
+      <c r="E29" s="4" t="n"/>
+      <c r="F29" s="4" t="n"/>
+      <c r="G29" s="4" t="n"/>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="99" t="inlineStr">
+        <is>
+          <t>LANCAMENTO</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="n"/>
+      <c r="C30" s="89" t="inlineStr">
+        <is>
+          <t>Produto em ramp-up — commercial_score_v2 pode estar subestimado (estoque incompleto)</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="n"/>
+      <c r="E30" s="4" t="n"/>
+      <c r="F30" s="4" t="n"/>
+      <c r="G30" s="4" t="n"/>
+    </row>
+    <row r="31" ht="6" customHeight="1"/>
+    <row r="32" ht="26" customHeight="1">
+      <c r="A32" s="87" t="inlineStr">
+        <is>
+          <t>TENDÊNCIA  ·  Reversas últimos 3 meses vs 3 meses anteriores</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="100" t="inlineStr">
+        <is>
+          <t>Aumentou</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="n"/>
+      <c r="C33" s="89" t="inlineStr">
+        <is>
+          <t>Reversas acelerando — urgência aumentada</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="n"/>
+      <c r="E33" s="4" t="n"/>
+      <c r="F33" s="4" t="n"/>
+      <c r="G33" s="4" t="n"/>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="101" t="inlineStr">
         <is>
           <t>Estável</t>
         </is>
       </c>
-      <c r="B24" s="4" t="n"/>
-      <c r="C24" s="89" t="inlineStr">
+      <c r="B34" s="4" t="n"/>
+      <c r="C34" s="89" t="inlineStr">
         <is>
           <t>Sem variação relevante</t>
         </is>
       </c>
-      <c r="D24" s="4" t="n"/>
-      <c r="E24" s="4" t="n"/>
-      <c r="F24" s="4" t="n"/>
-      <c r="G24" s="4" t="n"/>
-    </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="102" t="inlineStr">
+      <c r="D34" s="4" t="n"/>
+      <c r="E34" s="4" t="n"/>
+      <c r="F34" s="4" t="n"/>
+      <c r="G34" s="4" t="n"/>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="102" t="inlineStr">
         <is>
           <t>Caiu</t>
         </is>
       </c>
-      <c r="B25" s="4" t="n"/>
-      <c r="C25" s="89" t="inlineStr">
+      <c r="B35" s="4" t="n"/>
+      <c r="C35" s="89" t="inlineStr">
         <is>
           <t>Problema pode estar se resolvendo naturalmente</t>
         </is>
       </c>
-      <c r="D25" s="4" t="n"/>
-      <c r="E25" s="4" t="n"/>
-      <c r="F25" s="4" t="n"/>
-      <c r="G25" s="4" t="n"/>
+      <c r="D35" s="4" t="n"/>
+      <c r="E35" s="4" t="n"/>
+      <c r="F35" s="4" t="n"/>
+      <c r="G35" s="4" t="n"/>
+    </row>
+    <row r="36" ht="6" customHeight="1"/>
+    <row r="37" ht="26" customHeight="1">
+      <c r="A37" s="87" t="inlineStr">
+        <is>
+          <t>GLOSSÁRIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="108" t="inlineStr">
+        <is>
+          <t>T&amp;D</t>
+        </is>
+      </c>
+      <c r="B38" s="109" t="inlineStr">
+        <is>
+          <t>Trocas e Devoluções — evento de reversa gerado pelo cliente via Troquecommerce</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="n"/>
+      <c r="D38" s="4" t="n"/>
+      <c r="E38" s="4" t="n"/>
+      <c r="F38" s="4" t="n"/>
+      <c r="G38" s="4" t="n"/>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="108" t="inlineStr">
+        <is>
+          <t>td_rate</t>
+        </is>
+      </c>
+      <c r="B39" s="109" t="inlineStr">
+        <is>
+          <t>itens_retornados ÷ itens_vendidos — taxa bruta de T&amp;D do produto</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="n"/>
+      <c r="D39" s="4" t="n"/>
+      <c r="E39" s="4" t="n"/>
+      <c r="F39" s="4" t="n"/>
+      <c r="G39" s="4" t="n"/>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="108" t="inlineStr">
+        <is>
+          <t>delta_vs_categoria</t>
+        </is>
+      </c>
+      <c r="B40" s="109" t="inlineStr">
+        <is>
+          <t>td_rate_produto − td_rate_categoria — quanto o produto supera o benchmark da categoria</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="n"/>
+      <c r="D40" s="4" t="n"/>
+      <c r="E40" s="4" t="n"/>
+      <c r="F40" s="4" t="n"/>
+      <c r="G40" s="4" t="n"/>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="108" t="inlineStr">
+        <is>
+          <t>sell_through_Nd</t>
+        </is>
+      </c>
+      <c r="B41" s="109" t="inlineStr">
+        <is>
+          <t>% do estoque inicial vendido em N dias após lançamento — mede velocidade comercial real</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="n"/>
+      <c r="D41" s="4" t="n"/>
+      <c r="E41" s="4" t="n"/>
+      <c r="F41" s="4" t="n"/>
+      <c r="G41" s="4" t="n"/>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="108" t="inlineStr">
+        <is>
+          <t>mc3_ratio</t>
+        </is>
+      </c>
+      <c r="B42" s="109" t="inlineStr">
+        <is>
+          <t>Margem de contribuição nível 3 — contribuição econômica do produto após custos de marketing</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="n"/>
+      <c r="D42" s="4" t="n"/>
+      <c r="E42" s="4" t="n"/>
+      <c r="F42" s="4" t="n"/>
+      <c r="G42" s="4" t="n"/>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="108" t="inlineStr">
+        <is>
+          <t>td_score</t>
+        </is>
+      </c>
+      <c r="B43" s="109" t="inlineStr">
+        <is>
+          <t>Score composto de dor do cliente (0–1, CUME_DIST)</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="n"/>
+      <c r="D43" s="4" t="n"/>
+      <c r="E43" s="4" t="n"/>
+      <c r="F43" s="4" t="n"/>
+      <c r="G43" s="4" t="n"/>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="108" t="inlineStr">
+        <is>
+          <t>commercial_score_v2</t>
+        </is>
+      </c>
+      <c r="B44" s="109" t="inlineStr">
+        <is>
+          <t>Score composto de tração comercial + margem — versão 2 com sell-through e MC3 (0–1, CUME_DIST)</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="n"/>
+      <c r="D44" s="4" t="n"/>
+      <c r="E44" s="4" t="n"/>
+      <c r="F44" s="4" t="n"/>
+      <c r="G44" s="4" t="n"/>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="108" t="inlineStr">
+        <is>
+          <t>priority_score</t>
+        </is>
+      </c>
+      <c r="B45" s="109" t="inlineStr">
+        <is>
+          <t>0,50 × td_score + 0,50 × commercial_score_v2 — ranking global de urgência</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="n"/>
+      <c r="D45" s="4" t="n"/>
+      <c r="E45" s="4" t="n"/>
+      <c r="F45" s="4" t="n"/>
+      <c r="G45" s="4" t="n"/>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="108" t="inlineStr">
+        <is>
+          <t>sinal_priorizacao</t>
+        </is>
+      </c>
+      <c r="B46" s="109" t="inlineStr">
+        <is>
+          <t>Farol operacional de 5 buckets — gerado em SQL</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="n"/>
+      <c r="D46" s="4" t="n"/>
+      <c r="E46" s="4" t="n"/>
+      <c r="F46" s="4" t="n"/>
+      <c r="G46" s="4" t="n"/>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="108" t="inlineStr">
+        <is>
+          <t>sinal_kill_keep</t>
+        </is>
+      </c>
+      <c r="B47" s="109" t="inlineStr">
+        <is>
+          <t>Decisão estratégica de 2 estados — gerado em Python</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="n"/>
+      <c r="D47" s="4" t="n"/>
+      <c r="E47" s="4" t="n"/>
+      <c r="F47" s="4" t="n"/>
+      <c r="G47" s="4" t="n"/>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="108" t="inlineStr">
+        <is>
+          <t>pct_top_3_total</t>
+        </is>
+      </c>
+      <c r="B48" s="109" t="inlineStr">
+        <is>
+          <t>% das reversas tagueadas que os 3 principais motivos representam — alavanca potencial</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="n"/>
+      <c r="D48" s="4" t="n"/>
+      <c r="E48" s="4" t="n"/>
+      <c r="F48" s="4" t="n"/>
+      <c r="G48" s="4" t="n"/>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="108" t="inlineStr">
+        <is>
+          <t>CUME_DIST</t>
+        </is>
+      </c>
+      <c r="B49" s="109" t="inlineStr">
+        <is>
+          <t>Função SQL que calcula o percentil relativo de um valor dentro do portfólio (0 a 1)</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="n"/>
+      <c r="D49" s="4" t="n"/>
+      <c r="E49" s="4" t="n"/>
+      <c r="F49" s="4" t="n"/>
+      <c r="G49" s="4" t="n"/>
+    </row>
+    <row r="50" ht="20" customHeight="1">
+      <c r="A50" s="108" t="inlineStr">
+        <is>
+          <t>Cluster</t>
+        </is>
+      </c>
+      <c r="B50" s="109" t="inlineStr">
+        <is>
+          <t>Posicionamento estratégico: Hero · Core · Long tail · KILL · Lancamento · Breakthrough</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="n"/>
+      <c r="D50" s="4" t="n"/>
+      <c r="E50" s="4" t="n"/>
+      <c r="F50" s="4" t="n"/>
+      <c r="G50" s="4" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="37">
-    <mergeCell ref="A24:B24"/>
+  <mergeCells count="65">
+    <mergeCell ref="A32:G32"/>
+    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="C30:G30"/>
+    <mergeCell ref="C34:G34"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="B42:G42"/>
     <mergeCell ref="C6:G6"/>
-    <mergeCell ref="C24:G24"/>
     <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A22:G22"/>
+    <mergeCell ref="C15:G15"/>
+    <mergeCell ref="C33:G33"/>
+    <mergeCell ref="A20:G20"/>
     <mergeCell ref="C5:G5"/>
+    <mergeCell ref="B44:G44"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A10:G10"/>
+    <mergeCell ref="C26:G26"/>
+    <mergeCell ref="B38:G38"/>
+    <mergeCell ref="C29:G29"/>
     <mergeCell ref="C4:G4"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="C20:G20"/>
+    <mergeCell ref="C35:G35"/>
     <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="C16:G16"/>
-    <mergeCell ref="C25:G25"/>
-    <mergeCell ref="A15:G15"/>
-    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="B49:G49"/>
+    <mergeCell ref="B40:G40"/>
+    <mergeCell ref="C22:G22"/>
+    <mergeCell ref="A27:B27"/>
     <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="C21:G21"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="C12:G12"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="B45:G45"/>
+    <mergeCell ref="B41:G41"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="C11:G11"/>
+    <mergeCell ref="C27:G27"/>
+    <mergeCell ref="B50:G50"/>
+    <mergeCell ref="A16:G16"/>
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="A23:B23"/>
     <mergeCell ref="C23:G23"/>
     <mergeCell ref="C8:G8"/>
     <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A25:G25"/>
+    <mergeCell ref="A22:B22"/>
     <mergeCell ref="C17:G17"/>
+    <mergeCell ref="A35:B35"/>
     <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A37:G37"/>
+    <mergeCell ref="B47:G47"/>
     <mergeCell ref="C7:G7"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="B46:G46"/>
     <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="C28:G28"/>
     <mergeCell ref="A13:B13"/>
-    <mergeCell ref="C19:G19"/>
+    <mergeCell ref="B43:G43"/>
     <mergeCell ref="C13:G13"/>
-    <mergeCell ref="C18:G18"/>
+    <mergeCell ref="B48:G48"/>
+    <mergeCell ref="B39:G39"/>
+    <mergeCell ref="A34:B34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>